<commit_message>
doc: complete testing for modules 4 and 5
</commit_message>
<xml_diff>
--- a/Tests/excel/module03_test_cases.xlsx
+++ b/Tests/excel/module03_test_cases.xlsx
@@ -48,13 +48,19 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0064748B"/>
+      <color rgb="00137333"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00A50E0E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -73,12 +79,6 @@
       <name val="Segoe UI"/>
       <i val="1"/>
       <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00137333"/>
       <sz val="10"/>
     </font>
     <font>
@@ -145,8 +145,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00E6F4EA"/>
+        <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
     <fill>
@@ -163,6 +163,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FEF7E0"/>
         <bgColor rgb="00FEF7E0"/>
       </patternFill>
@@ -171,12 +177,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2E8F0"/>
         <bgColor rgb="00E2E8F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E6F4EA"/>
-        <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -252,24 +252,27 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -288,10 +291,10 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -306,19 +309,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -896,354 +899,354 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Module 03 - Feature &amp; Priority Summary Report</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Summary of test cases per feature, calculated via Excel formulas</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Total Features</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Total Test Cases</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>High Priority Features</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Medium Priority Features</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Low Priority Features</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="14">
+      <c r="A5" s="15">
         <f>COUNTA(A9:A16)</f>
         <v/>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="16">
         <f>F17</f>
         <v/>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="17">
         <f>COUNTIF(C9:C16, "&gt;0")</f>
         <v/>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="18">
         <f>COUNTIFS(C9:C16, 0, D9:D16, "&gt;0")</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>COUNTIFS(C9:C16, 0, D9:D16, 0, E9:E16, "&gt;0")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Feature Categorization &amp; Priority Breakdown</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Feature ID</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Feature Name</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>High Priority</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Medium Priority</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>Low Priority</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>Total TCs</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>M03-F01</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Course / Subject Creation</t>
         </is>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="25">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A9, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="26">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A9, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="27">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A9, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="28">
         <f>SUM(C9:E9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>M03-F02</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
         <is>
           <t>Grade Entry Structure</t>
         </is>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="31">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A10, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="32">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A10, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="33">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A10, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="34">
         <f>SUM(C10:E10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>M03-F03</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Automatic TBKT Calculation</t>
         </is>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="25">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A11, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="26">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A11, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="27">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A11, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="28">
         <f>SUM(C11:E11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>M03-F04</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>Grade Upload via CSV</t>
         </is>
       </c>
-      <c r="C12" s="30">
+      <c r="C12" s="31">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A12, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="32">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A12, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="33">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A12, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F12" s="33">
+      <c r="F12" s="34">
         <f>SUM(C12:E12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>M03-F07</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Manual GPA &amp; Letter Grade Entry</t>
         </is>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="25">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A13, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="26">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A13, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="27">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A13, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="28">
         <f>SUM(C13:E13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>M03-F05</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Subject Deletion</t>
         </is>
       </c>
-      <c r="C14" s="30">
+      <c r="C14" s="31">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A14, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D14" s="31">
+      <c r="D14" s="32">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A14, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="33">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A14, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F14" s="33">
+      <c r="F14" s="34">
         <f>SUM(C14:E14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>M03-F06</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>PDF Transcript Export</t>
         </is>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="25">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A15, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="26">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A15, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="27">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A15, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="28">
         <f>SUM(C15:E15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>M03-SEC</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Access Control &amp; Security</t>
         </is>
       </c>
-      <c r="C16" s="30">
+      <c r="C16" s="31">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A16, 'Module03'!$N$2:$N$23, "High")</f>
         <v/>
       </c>
-      <c r="D16" s="31">
+      <c r="D16" s="32">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A16, 'Module03'!$N$2:$N$23, "Medium")</f>
         <v/>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="33">
         <f>COUNTIFS('Module03'!$C$2:$C$23, A16, 'Module03'!$N$2:$N$23, "Low")</f>
         <v/>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="34">
         <f>SUM(C16:E16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="34" t="inlineStr">
+      <c r="A17" s="35" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B17" s="35">
+      <c r="B17" s="36">
         <f>COUNTA(A9:A16)&amp;" Features"</f>
         <v/>
       </c>
-      <c r="C17" s="34">
+      <c r="C17" s="35">
         <f>SUM(C9:C16)</f>
         <v/>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="35">
         <f>SUM(D9:D16)</f>
         <v/>
       </c>
-      <c r="E17" s="34">
+      <c r="E17" s="35">
         <f>SUM(E9:E16)</f>
         <v/>
       </c>
-      <c r="F17" s="34">
+      <c r="F17" s="35">
         <f>SUM(F9:F16)</f>
         <v/>
       </c>
@@ -1415,7 +1418,7 @@
       <c r="K2" s="4" t="inlineStr"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -1487,7 +1490,7 @@
       <c r="K3" s="9" t="inlineStr"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr"/>
@@ -1557,10 +1560,14 @@
           <t>Saving is blocked. Error message 'Subject Name is required' displays. Name field is highlighted in red.</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Hệ thống không thực hiện việc tạo môn học nhưng cũng không có thông báo nào cho người dùng.</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -1631,7 +1638,7 @@
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1703,7 +1710,7 @@
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1775,7 +1782,7 @@
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1847,7 +1854,7 @@
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1919,7 +1926,7 @@
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1990,7 +1997,7 @@
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2062,7 +2069,7 @@
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2133,7 +2140,7 @@
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2204,7 +2211,7 @@
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr"/>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2273,7 +2280,7 @@
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2346,7 +2353,7 @@
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2417,7 +2424,7 @@
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L16" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2489,7 +2496,7 @@
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2561,7 +2568,7 @@
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="5" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2633,7 +2640,7 @@
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2704,13 +2711,13 @@
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L20" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="10" t="inlineStr">
+      <c r="N20" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2775,13 +2782,13 @@
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L21" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr"/>
-      <c r="N21" s="10" t="inlineStr">
+      <c r="N21" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2846,7 +2853,7 @@
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr">
+      <c r="L22" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2917,7 +2924,7 @@
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="L23" s="10" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>

</xml_diff>